<commit_message>
detection des cases et mise à jour des feuilles de marquage
</commit_message>
<xml_diff>
--- a/externe/FeuilleMarquage.xlsx
+++ b/externe/FeuilleMarquage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nathan\Documents\Projet\IABelote\externe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3B1608-CD68-444B-8B78-79F7B4302DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730060AE-2DBD-430E-BEAE-0536667EA8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5130" yWindow="3795" windowWidth="19200" windowHeight="10080" xr2:uid="{5939A16A-11FD-4A6D-A599-6DB9184D917B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{5939A16A-11FD-4A6D-A599-6DB9184D917B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -41,16 +41,10 @@
     <t>Equipe 1</t>
   </si>
   <si>
-    <t>Nom prenom</t>
-  </si>
-  <si>
     <t>Equipe 2</t>
   </si>
   <si>
     <t>N pli</t>
-  </si>
-  <si>
-    <t>N equipe preneuse</t>
   </si>
   <si>
     <t>Point</t>
@@ -63,6 +57,12 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>prenom</t>
   </si>
 </sst>
 </file>
@@ -110,7 +110,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -145,6 +145,191 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -154,22 +339,44 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Entrée" xfId="1" builtinId="20"/>
@@ -506,207 +713,187 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E9E8F3A-6113-49F4-BB0B-E4FA83D3EFA9}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:G18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="7" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" customWidth="1"/>
+    <col min="3" max="7" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="8"/>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="2:7" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="2:7" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="2:7" s="1" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5"/>
+    </row>
+    <row r="6" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="6">
         <v>1</v>
       </c>
-      <c r="F1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="3" t="s">
+      <c r="C6" s="14"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="4">
         <v>2</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="C7" s="15"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C8" s="15"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="4">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C9" s="15"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="4">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="C10" s="15"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="4">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="C11" s="15"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="4">
         <v>7</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="C12" s="15"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="4">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
-        <v>1</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="6"/>
-    </row>
-    <row r="7" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>2</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>3</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>4</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>5</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
+      <c r="C13" s="15"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="4">
+        <v>9</v>
+      </c>
+      <c r="C14" s="15"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="4">
+        <v>10</v>
+      </c>
+      <c r="C15" s="15"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="4">
+        <v>11</v>
+      </c>
+      <c r="C16" s="15"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="2:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="4">
+        <v>12</v>
+      </c>
+      <c r="C17" s="15"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="2:6" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="6"/>
-    </row>
-    <row r="12" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
-        <v>7</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="6"/>
-    </row>
-    <row r="13" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>8</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="6"/>
-    </row>
-    <row r="14" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
-        <v>9</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
-        <v>10</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="6"/>
-    </row>
-    <row r="16" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
-        <v>11</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="6"/>
-    </row>
-    <row r="17" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
-        <v>12</v>
-      </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="6"/>
-    </row>
-    <row r="18" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>